<commit_message>
Finalize D4 common-support validation
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D4 Parallel-redundancy Temporal Consistency/outputs/data/D4_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D4 Parallel-redundancy Temporal Consistency/outputs/data/D4_audit_log.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,7 +454,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>D4V14_20260726_100717</t>
+          <t>D4V15_20260813_033216</t>
         </is>
       </c>
     </row>
@@ -466,7 +466,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>d4-v1.4-canonical-d4-20260726</t>
+          <t>d4-v1.5-common-support-frozen-d4-20260813</t>
         </is>
       </c>
     </row>
@@ -478,127 +478,215 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>D4CAL-V14-7a16d7f511d3</t>
+          <t>D4CAL-V15-f6c351de01b0</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>generated_utc</t>
+          <t>fit_phase</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-26T10:09:22.480272+00:00</t>
+          <t>development</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>d2_run_id</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>D2V1_20260722_1714</t>
-        </is>
+          <t>fit_start</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>45870</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>d2_calibration_id</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>NorthBank_D2_v1_20260722</t>
-        </is>
+          <t>fit_end</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>46046.99998842592</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>n_rows</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>42847</v>
+          <t>internal_validation_start</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>46054</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>n_pairs</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>7</v>
+          <t>internal_validation_end</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>46125.99998842592</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>data_start</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>45870</v>
+          <t>terminal_status</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>pending_genuinely_unseen_future_period</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>data_end</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>46125.99305555555</v>
+          <t>common_support_policy</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>synchronous_timestamp_primary</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>evaluable_rate_D4_raw</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.8865731556468364</v>
+          <t>distribution_component_version</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>full_w1_0.60_ks_0.40_development_frozen</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>D4_forDQR_status</t>
+          <t>generated_utc</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>provisional only; pending D5 arbitration</t>
+          <t>2026-08-13T03:43:43.929931+00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>benchmark_D5_screen</t>
+          <t>d2_run_id</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>pending; no D5 proxy generated</t>
+          <t>D2V4_20260805_1127</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>d2_calibration_id</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NorthBank_D2_v4_20260805</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>n_rows</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>42847</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>n_pairs</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>data_start</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>45870</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>data_end</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>46125.99305555555</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>evaluable_rate_D4_raw</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.9888907041333116</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>D4_forDQR_status</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>provisional only; pending D5 arbitration</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>benchmark_D5_screen</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>pending; no D5 proxy generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>causal_claim</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>pair asymmetry only; sensor/process cause pending D5</t>
         </is>
@@ -702,7 +790,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-26T10:03:42.151123+00:00</t>
+          <t>2026-07-27T08:02:48.122703+00:00</t>
         </is>
       </c>
     </row>
@@ -724,7 +812,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-26T10:03:50.930617+00:00</t>
+          <t>2026-07-27T08:02:48.137757+00:00</t>
         </is>
       </c>
     </row>
@@ -741,12 +829,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>70a4a093f0900b090d49dbe8eda8a025e5eb840fce44a267f43636627029c08a</t>
+          <t>ac051d9a24a17523433c63187cf63f0128efb185325a1ea789633f7fc13d04a6</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-22T09:14:38.920336+00:00</t>
+          <t>2026-08-05T03:28:59.791070+00:00</t>
         </is>
       </c>
     </row>
@@ -763,12 +851,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>00722ca5647d83d906091cecba1bf6904ae93871102766d556416226153c73d7</t>
+          <t>9ab231ea9d1bd72ba6f74b8a30198fb6af41bc1796d5236f1fd864d482e73121</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-26T09:43:55.829080+00:00</t>
+          <t>2026-08-13T02:48:32.783588+00:00</t>
         </is>
       </c>
     </row>
@@ -785,12 +873,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>f6b9f6de7d5159494bd45de3a04f3a57537869e4d2c70a0af8192fba77a0e58e</t>
+          <t>7cdd93fbd646fbfc9b7ac14411fcc3bc95b7cc5b05b32de29422275022d77f19</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-26T09:51:14.227894+00:00</t>
+          <t>2026-08-13T03:31:36.648093+00:00</t>
         </is>
       </c>
     </row>
@@ -807,12 +895,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ddef43ff2e7d872c5c7a30e6485e7b856d058a96b800854fe40ac815a5b48120</t>
+          <t>1f7845876b73515ea34171dd34a50d279aa32d0fd3244226b8ab9774292f4bfe</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-26T08:43:40.442735+00:00</t>
+          <t>2026-08-13T02:48:32.786982+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harden D4 dependence-aware inference
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D4 Parallel-redundancy Temporal Consistency/outputs/data/D4_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D4 Parallel-redundancy Temporal Consistency/outputs/data/D4_audit_log.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>D4V15_20260813_033216</t>
+          <t>D4V151_20260813_083347</t>
         </is>
       </c>
     </row>
@@ -466,7 +466,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>d4-v1.5-common-support-frozen-d4-20260813</t>
+          <t>d4-v1.5.1-statistical-dependence-audit-20260813</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>D4CAL-V15-f6c351de01b0</t>
+          <t>D4CAL-V151-66fe1bb6b7d3</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-13T03:43:43.929931+00:00</t>
+          <t>2026-08-13T08:36:22.471481+00:00</t>
         </is>
       </c>
     </row>
@@ -851,12 +851,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>9ab231ea9d1bd72ba6f74b8a30198fb6af41bc1796d5236f1fd864d482e73121</t>
+          <t>213ecde94309486e5a09659e2306c3028459cc77786e175b98e381cba198df74</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-08-13T02:48:32.783588+00:00</t>
+          <t>2026-08-13T08:26:25.369829+00:00</t>
         </is>
       </c>
     </row>
@@ -873,12 +873,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>7cdd93fbd646fbfc9b7ac14411fcc3bc95b7cc5b05b32de29422275022d77f19</t>
+          <t>4c9dfbaa3c0068d0476fd8a2f6a1602802bacb31bb9c6c60f5bf7dfa0f79c5a6</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-08-13T03:31:36.648093+00:00</t>
+          <t>2026-08-13T08:33:10.776586+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>